<commit_message>
Final gap check fixes: page states under the header, clear publish buttons, one exam slot per campus per day, pay-by deadline, In review wording, Prepare PDFs in the flows, 2026-layout Excel template, docs aligned
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mockups/docs/tpt-scores-template.xlsx
+++ b/mockups/docs/tpt-scores-template.xlsx
@@ -51,7 +51,9 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,162 +419,292 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:X3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="17" customWidth="1" min="16" max="16"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>examinee_no</t>
+          <t>Name of Examinee</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>Examinee Number</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>english_ss</t>
+          <t>Preferred Program</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>english_stanine</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>science_ss</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>science_stanine</t>
-        </is>
-      </c>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>math_ss</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>math_stanine</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>filipino_ss</t>
-        </is>
-      </c>
+          <t>Science</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>filipino_stanine</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>social_studies_ss</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>social_studies_stanine</t>
-        </is>
-      </c>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>esm_ss</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>esm_stanine</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>overall_ss</t>
-        </is>
-      </c>
+          <t>Filipino</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>overall_stanine</t>
-        </is>
-      </c>
+          <t>Social Studies</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="n"/>
+      <c r="R1" s="1" t="n"/>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>ESM Competency Score</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Overall Score</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="n"/>
+      <c r="X1" s="1" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>500214</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Dela Cruz, Maria Santos</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Standard Score</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Stanine</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Qualitative Interpretation</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Standard Score</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>Stanine</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>Qualitative Interpretation</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>Standard Score</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>Stanine</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>Qualitative Interpretation</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>Standard Score</t>
+        </is>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t>Stanine</t>
+        </is>
+      </c>
+      <c r="O2" s="1" t="inlineStr">
+        <is>
+          <t>Qualitative Interpretation</t>
+        </is>
+      </c>
+      <c r="P2" s="1" t="inlineStr">
+        <is>
+          <t>Standard Score</t>
+        </is>
+      </c>
+      <c r="Q2" s="1" t="inlineStr">
+        <is>
+          <t>Stanine</t>
+        </is>
+      </c>
+      <c r="R2" s="1" t="inlineStr">
+        <is>
+          <t>Qualitative Interpretation</t>
+        </is>
+      </c>
+      <c r="S2" s="1" t="inlineStr">
+        <is>
+          <t>Standard Score</t>
+        </is>
+      </c>
+      <c r="T2" s="1" t="inlineStr">
+        <is>
+          <t>Stanine</t>
+        </is>
+      </c>
+      <c r="U2" s="1" t="inlineStr">
+        <is>
+          <t>Qualitative Interpretation</t>
+        </is>
+      </c>
+      <c r="V2" s="1" t="inlineStr">
+        <is>
+          <t>Standard Score</t>
+        </is>
+      </c>
+      <c r="W2" s="1" t="inlineStr">
+        <is>
+          <t>Stanine</t>
+        </is>
+      </c>
+      <c r="X2" s="1" t="inlineStr">
+        <is>
+          <t>Qualitative Interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DELA CRUZ, MARIA SANTOS (SAMPLE)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>500214</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Isulan-BS Civil Engineering</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>612</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E3" t="n">
         <v>8</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Above Average</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
         <v>548</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H3" t="n">
         <v>6</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
         <v>571</v>
       </c>
-      <c r="H2" t="n">
+      <c r="K3" t="n">
         <v>7</v>
       </c>
-      <c r="I2" t="n">
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Above Average</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
         <v>655</v>
       </c>
-      <c r="J2" t="n">
+      <c r="N3" t="n">
         <v>9</v>
       </c>
-      <c r="K2" t="n">
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Outstanding</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
         <v>530</v>
       </c>
-      <c r="L2" t="n">
+      <c r="Q3" t="n">
         <v>6</v>
       </c>
-      <c r="M2" t="n">
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
         <v>566</v>
       </c>
-      <c r="N2" t="n">
+      <c r="T3" t="n">
         <v>7</v>
       </c>
-      <c r="O2" t="n">
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Above Average</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
         <v>584</v>
       </c>
-      <c r="P2" t="n">
+      <c r="W3" t="n">
         <v>7</v>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Above Average</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="J1:L1"/>
+    <mergeCell ref="P1:R1"/>
+    <mergeCell ref="S1:U1"/>
+    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="V1:X1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>